<commit_message>
Question images: in the Excel sheet and from the admin panel
- New "صورة السؤال" column; pictures pasted over a row are attached by column:
  question / each option (image-only options allowed) / explanation
- Images stored in Postgres (question_media), type checked by file signature, 2MB each
- Served at /api/media/q/<id>/<slot>/<hash> (unguessable, cached immutably)
- Shown in practice, mistakes retry, competitions (options shuffled with their images),
  explanations and competition review; sent to Gemini with the question
- Admin question window: upload/replace/delete per slot with preview; large photos
  are shrunk in the browser before upload
- Template includes examples (triangle question image, graph options)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012XR2U4cqX9ftZsGm1WFMS8
</commit_message>
<xml_diff>
--- a/templates/questions-template.xlsx
+++ b/templates/questions-template.xlsx
@@ -11,11 +11,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="78">
   <si>
     <t>السؤال</t>
   </si>
   <si>
+    <t>صورة السؤال</t>
+  </si>
+  <si>
     <t>أ</t>
   </si>
   <si>
@@ -55,6 +58,9 @@
     <t>جسم كتلته 2 كجم يتحرك بعجلة 3 م/ث². ما القوة المؤثرة عليه؟</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>5 نيوتن</t>
   </si>
   <si>
@@ -85,9 +91,6 @@
     <t>درس</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>وحدة قياس الشغل هي:</t>
   </si>
   <si>
@@ -212,6 +215,36 @@
   </si>
   <si>
     <t>مسائل</t>
+  </si>
+  <si>
+    <t>من الشكل: احسب طول الوتر في المثلث القائم.</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>فيثاغورس: الوتر² = 3² + 4² = 25 ← الوتر = 5</t>
+  </si>
+  <si>
+    <t>الوتر² = ضلع² + ضلع²</t>
+  </si>
+  <si>
+    <t>نظرية فيثاغورس</t>
+  </si>
+  <si>
+    <t>أي من الرسومات البيانية التالية يمثل علاقة طردية؟</t>
+  </si>
+  <si>
+    <t>العلاقة الطردية خط مستقيم يمر بنقطة الأصل</t>
+  </si>
+  <si>
+    <t>ص = ك × س</t>
+  </si>
+  <si>
+    <t>التناسب</t>
   </si>
 </sst>
 </file>
@@ -268,6 +301,206 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28000</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>119999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1524000" cy="1047750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>22000</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>89999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1047750" cy="781050"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>22000</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>89999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1047750" cy="781050"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>21999</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>89999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1047750" cy="781050"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>21999</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>89999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1047750" cy="781050"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -592,21 +825,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
-    <col min="2" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="40" customWidth="1"/>
-    <col min="8" max="8" width="30" customWidth="1"/>
-    <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
-    <col min="11" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="40" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="12" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -646,54 +880,60 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F2" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="H2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="L2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M2" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="N2" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
         <v>27</v>
@@ -705,36 +945,39 @@
         <v>29</v>
       </c>
       <c r="F3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="G3" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="H3" t="s">
         <v>31</v>
       </c>
       <c r="I3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="J3" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="K3" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="L3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M3" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="N3" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
         <v>35</v>
@@ -749,16 +992,16 @@
         <v>38</v>
       </c>
       <c r="G4" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="H4" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="I4" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="J4" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="K4" t="s">
         <v>40</v>
@@ -769,13 +1012,16 @@
       <c r="M4" t="s">
         <v>42</v>
       </c>
+      <c r="N4" t="s">
+        <v>43</v>
+      </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
         <v>45</v>
@@ -787,36 +1033,39 @@
         <v>47</v>
       </c>
       <c r="F5" t="s">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="G5" t="s">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="H5" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="I5" t="s">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="J5" t="s">
         <v>50</v>
       </c>
       <c r="K5" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="L5" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="M5" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="N5" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
         <v>53</v>
@@ -828,36 +1077,39 @@
         <v>55</v>
       </c>
       <c r="F6" t="s">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="G6" t="s">
+        <v>4</v>
+      </c>
+      <c r="H6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" t="s">
+        <v>57</v>
+      </c>
+      <c r="J6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" t="s">
         <v>24</v>
       </c>
-      <c r="H6" t="s">
-        <v>56</v>
-      </c>
-      <c r="I6" t="s">
-        <v>49</v>
-      </c>
-      <c r="J6" t="s">
-        <v>57</v>
-      </c>
-      <c r="K6" t="s">
-        <v>22</v>
-      </c>
-      <c r="L6" t="s">
-        <v>41</v>
-      </c>
       <c r="M6" t="s">
-        <v>58</v>
+        <v>42</v>
+      </c>
+      <c r="N6" t="s">
+        <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B7" t="s">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
         <v>61</v>
@@ -869,16 +1121,16 @@
         <v>63</v>
       </c>
       <c r="F7" t="s">
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="G7" t="s">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="H7" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="I7" t="s">
-        <v>64</v>
+        <v>15</v>
       </c>
       <c r="J7" t="s">
         <v>65</v>
@@ -887,14 +1139,106 @@
         <v>66</v>
       </c>
       <c r="L7" t="s">
-        <v>23</v>
+        <v>67</v>
       </c>
       <c r="M7" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="N7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" ht="120" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E8" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" t="s">
+        <v>2</v>
+      </c>
+      <c r="H8" t="s">
+        <v>71</v>
+      </c>
+      <c r="I8" t="s">
+        <v>72</v>
+      </c>
+      <c r="J8" t="s">
+        <v>65</v>
+      </c>
+      <c r="K8" t="s">
+        <v>73</v>
+      </c>
+      <c r="L8" t="s">
+        <v>67</v>
+      </c>
+      <c r="M8" t="s">
+        <v>25</v>
+      </c>
+      <c r="N8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" t="s">
+        <v>2</v>
+      </c>
+      <c r="H9" t="s">
+        <v>75</v>
+      </c>
+      <c r="I9" t="s">
+        <v>76</v>
+      </c>
+      <c r="J9" t="s">
+        <v>65</v>
+      </c>
+      <c r="K9" t="s">
+        <v>77</v>
+      </c>
+      <c r="L9" t="s">
+        <v>67</v>
+      </c>
+      <c r="M9" t="s">
+        <v>25</v>
+      </c>
+      <c r="N9" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>